<commit_message>
docs: carry today's behaviour changes into every public document
A sweep of the public docs against the day's changes found them missing in
several places:

- Auto-denial only with the consent store on (F-251): README (section and
  table), sgtmClient/README (flow step 5, auto_deny_load_gtm), PRIVACY-
  DATAFLOW (two places), SESSION-REDESIGN (two places).
- README: when the auto-denial preset masks a decision the CMP already
  holds, and that useListener / no store URL / consent_poll_ms 0 mean no
  poll lifts it (a manual call_cc() does not either).
- cmp/README-cmp: a blocked Consentmanager is no decision (F-164).
- EVENTS.md and its xlsx twin: no "JS Error" events with jsErrors: false.
  Only one cell of the v1.5 workbook changed (compared cell by cell
  against HEAD); the v1.4 workbook is untouched.
- configurator/README: version 2.2.1, jsErrors in step 6.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/aGTM-Events-v1.5.xlsx
+++ b/assets/aGTM-Events-v1.5.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="aGTM Events" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Page &amp; Device Info" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="aGTM Variables" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="aGTM Events" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Page &amp; Device Info" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="aGTM Variables" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Legend" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>ONLY on "JS Error": error counter (max. 5 are pushed, 100 counted)</t>
+          <t>ONLY on "JS Error": error counter (max. 5 are pushed, 100 counted); no "JS Error" events with jsErrors: false</t>
         </is>
       </c>
       <c r="Q12" s="5" t="inlineStr">

</xml_diff>